<commit_message>
update: crawl data 19/8
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -9686,7 +9686,7 @@
         <v>46252.02187171296</v>
       </c>
       <c r="F4" s="180" t="n">
-        <v>46252.7212319852</v>
+        <v>46252.72123199074</v>
       </c>
       <c r="G4" s="181">
         <f>IF(OR(E4="",F4=""),"",(F4-E4)*24)</f>
@@ -9736,27 +9736,56 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E5" s="180" t="n"/>
-      <c r="F5" s="180" t="n"/>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E5" s="180" t="n">
+        <v>46253.02209534722</v>
+      </c>
+      <c r="F5" s="180" t="n">
+        <v>46253.72352921589</v>
+      </c>
       <c r="G5" s="181">
         <f>IF(OR(E5="",F5=""),"",(F5-E5)*24)</f>
         <v/>
       </c>
-      <c r="H5" s="182" t="n"/>
-      <c r="I5" s="182" t="n"/>
-      <c r="J5" s="182" t="n"/>
-      <c r="K5" s="182" t="n"/>
-      <c r="L5" s="182" t="n"/>
-      <c r="M5" s="182" t="n"/>
-      <c r="N5" s="182" t="n"/>
-      <c r="O5" s="182" t="n"/>
+      <c r="H5" s="182" t="n">
+        <v>4260</v>
+      </c>
+      <c r="I5" s="182" t="n">
+        <v>4260</v>
+      </c>
+      <c r="J5" s="182" t="n">
+        <v>3816</v>
+      </c>
+      <c r="K5" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="182" t="n">
+        <v>444</v>
+      </c>
+      <c r="M5" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="182" t="n">
+        <v>39507</v>
+      </c>
       <c r="P5" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q5" s="86" t="n"/>
+      <c r="Q5" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 12 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="24" customHeight="1" s="80">
       <c r="A6" s="177" t="n">

</xml_diff>

<commit_message>
feat: update craw 21/8
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -9810,7 +9810,7 @@
         <v>46254.04391013889</v>
       </c>
       <c r="F6" s="180" t="n">
-        <v>46254.73005012742</v>
+        <v>46254.73005012731</v>
       </c>
       <c r="G6" s="181">
         <f>IF(OR(E6="",F6=""),"",(F6-E6)*24)</f>
@@ -9860,27 +9860,56 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E7" s="180" t="n"/>
-      <c r="F7" s="180" t="n"/>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="E7" s="180" t="n">
+        <v>46255.07475989583</v>
+      </c>
+      <c r="F7" s="180" t="n">
+        <v>46255.90631582349</v>
+      </c>
       <c r="G7" s="181">
         <f>IF(OR(E7="",F7=""),"",(F7-E7)*24)</f>
         <v/>
       </c>
-      <c r="H7" s="182" t="n"/>
-      <c r="I7" s="182" t="n"/>
-      <c r="J7" s="182" t="n"/>
-      <c r="K7" s="182" t="n"/>
-      <c r="L7" s="182" t="n"/>
-      <c r="M7" s="182" t="n"/>
-      <c r="N7" s="182" t="n"/>
-      <c r="O7" s="182" t="n"/>
+      <c r="H7" s="182" t="n">
+        <v>4260</v>
+      </c>
+      <c r="I7" s="182" t="n">
+        <v>4260</v>
+      </c>
+      <c r="J7" s="182" t="n">
+        <v>3808</v>
+      </c>
+      <c r="K7" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="182" t="n">
+        <v>452</v>
+      </c>
+      <c r="M7" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="182" t="n">
+        <v>34030</v>
+      </c>
       <c r="P7" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q7" s="86" t="n"/>
+      <c r="Q7" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 16 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="24" customHeight="1" s="80">
       <c r="A8" s="177" t="n">

</xml_diff>

<commit_message>
feat: update crawl 22/8
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -9872,7 +9872,7 @@
         <v>46255.07475989583</v>
       </c>
       <c r="F7" s="180" t="n">
-        <v>46255.90631582349</v>
+        <v>46255.90631582176</v>
       </c>
       <c r="G7" s="181">
         <f>IF(OR(E7="",F7=""),"",(F7-E7)*24)</f>
@@ -9922,27 +9922,56 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E8" s="180" t="n"/>
-      <c r="F8" s="180" t="n"/>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="E8" s="180" t="n">
+        <v>46256.02737123842</v>
+      </c>
+      <c r="F8" s="180" t="n">
+        <v>46256.69755518941</v>
+      </c>
       <c r="G8" s="181">
         <f>IF(OR(E8="",F8=""),"",(F8-E8)*24)</f>
         <v/>
       </c>
-      <c r="H8" s="182" t="n"/>
-      <c r="I8" s="182" t="n"/>
-      <c r="J8" s="182" t="n"/>
-      <c r="K8" s="182" t="n"/>
-      <c r="L8" s="182" t="n"/>
-      <c r="M8" s="182" t="n"/>
-      <c r="N8" s="182" t="n"/>
-      <c r="O8" s="182" t="n"/>
+      <c r="H8" s="182" t="n">
+        <v>4260</v>
+      </c>
+      <c r="I8" s="182" t="n">
+        <v>4260</v>
+      </c>
+      <c r="J8" s="182" t="n">
+        <v>3782</v>
+      </c>
+      <c r="K8" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="182" t="n">
+        <v>478</v>
+      </c>
+      <c r="M8" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="182" t="n">
+        <v>34252</v>
+      </c>
       <c r="P8" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q8" s="86" t="n"/>
+      <c r="Q8" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 17 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="24" customHeight="1" s="80">
       <c r="A9" s="177" t="n">

</xml_diff>

<commit_message>
feat: update crawl 23/8
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -9934,7 +9934,7 @@
         <v>46256.02737123842</v>
       </c>
       <c r="F8" s="180" t="n">
-        <v>46256.69755518941</v>
+        <v>46256.69755518519</v>
       </c>
       <c r="G8" s="181">
         <f>IF(OR(E8="",F8=""),"",(F8-E8)*24)</f>
@@ -9984,27 +9984,56 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E9" s="180" t="n"/>
-      <c r="F9" s="180" t="n"/>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="E9" s="180" t="n">
+        <v>46257.02248891204</v>
+      </c>
+      <c r="F9" s="180" t="n">
+        <v>46257.72114275934</v>
+      </c>
       <c r="G9" s="181">
         <f>IF(OR(E9="",F9=""),"",(F9-E9)*24)</f>
         <v/>
       </c>
-      <c r="H9" s="182" t="n"/>
-      <c r="I9" s="182" t="n"/>
-      <c r="J9" s="182" t="n"/>
-      <c r="K9" s="182" t="n"/>
-      <c r="L9" s="182" t="n"/>
-      <c r="M9" s="182" t="n"/>
-      <c r="N9" s="182" t="n"/>
-      <c r="O9" s="182" t="n"/>
+      <c r="H9" s="182" t="n">
+        <v>4260</v>
+      </c>
+      <c r="I9" s="182" t="n">
+        <v>4260</v>
+      </c>
+      <c r="J9" s="182" t="n">
+        <v>3818</v>
+      </c>
+      <c r="K9" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="182" t="n">
+        <v>430</v>
+      </c>
+      <c r="M9" s="182" t="n">
+        <v>12</v>
+      </c>
+      <c r="N9" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="182" t="n">
+        <v>34674</v>
+      </c>
       <c r="P9" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q9" s="86" t="n"/>
+      <c r="Q9" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 18 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="24" customHeight="1" s="80">
       <c r="A10" s="177" t="n">

</xml_diff>

<commit_message>
feat: create plan to merge database
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -9996,7 +9996,7 @@
         <v>46257.02248891204</v>
       </c>
       <c r="F9" s="180" t="n">
-        <v>46257.72114275934</v>
+        <v>46257.72114275463</v>
       </c>
       <c r="G9" s="181">
         <f>IF(OR(E9="",F9=""),"",(F9-E9)*24)</f>
@@ -10046,10 +10046,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E10" s="180" t="n"/>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E10" s="180" t="n">
+        <v>46258.02198333821</v>
+      </c>
       <c r="F10" s="180" t="n"/>
       <c r="G10" s="181">
         <f>IF(OR(E10="",F10=""),"",(F10-E10)*24)</f>
@@ -10066,7 +10073,11 @@
       <c r="P10" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q10" s="86" t="n"/>
+      <c r="Q10" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled crawl đã tạo durable run; save_artifacts=false</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="24" customHeight="1" s="80">
       <c r="A11" s="177" t="n">

</xml_diff>

<commit_message>
feat: update crawl 24/8
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -10046,36 +10046,54 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Đang chạy</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="E10" s="180" t="n">
-        <v>46258.02198333821</v>
-      </c>
-      <c r="F10" s="180" t="n"/>
+        <v>46258.03397636574</v>
+      </c>
+      <c r="F10" s="180" t="n">
+        <v>46258.71595146876</v>
+      </c>
       <c r="G10" s="181">
         <f>IF(OR(E10="",F10=""),"",(F10-E10)*24)</f>
         <v/>
       </c>
-      <c r="H10" s="182" t="n"/>
-      <c r="I10" s="182" t="n"/>
-      <c r="J10" s="182" t="n"/>
-      <c r="K10" s="182" t="n"/>
-      <c r="L10" s="182" t="n"/>
-      <c r="M10" s="182" t="n"/>
-      <c r="N10" s="182" t="n"/>
-      <c r="O10" s="182" t="n"/>
+      <c r="H10" s="182" t="n">
+        <v>4260</v>
+      </c>
+      <c r="I10" s="182" t="n">
+        <v>4260</v>
+      </c>
+      <c r="J10" s="182" t="n">
+        <v>3821</v>
+      </c>
+      <c r="K10" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="182" t="n">
+        <v>427</v>
+      </c>
+      <c r="M10" s="182" t="n">
+        <v>12</v>
+      </c>
+      <c r="N10" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="182" t="n">
+        <v>34218</v>
+      </c>
       <c r="P10" s="182" t="n">
         <v>12</v>
       </c>
       <c r="Q10" s="86" t="inlineStr">
         <is>
-          <t>Scheduled crawl đã tạo durable run; save_artifacts=false</t>
+          <t>Scheduled run 20 đã đạt terminal state</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: update crawl 25/8
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -10058,7 +10058,7 @@
         <v>46258.03397636574</v>
       </c>
       <c r="F10" s="180" t="n">
-        <v>46258.71595146876</v>
+        <v>46258.71595146991</v>
       </c>
       <c r="G10" s="181">
         <f>IF(OR(E10="",F10=""),"",(F10-E10)*24)</f>
@@ -10108,27 +10108,56 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E11" s="180" t="n"/>
-      <c r="F11" s="180" t="n"/>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="E11" s="180" t="n">
+        <v>46259.02196075232</v>
+      </c>
+      <c r="F11" s="180" t="n">
+        <v>46259.69631300233</v>
+      </c>
       <c r="G11" s="181">
         <f>IF(OR(E11="",F11=""),"",(F11-E11)*24)</f>
         <v/>
       </c>
-      <c r="H11" s="182" t="n"/>
-      <c r="I11" s="182" t="n"/>
-      <c r="J11" s="182" t="n"/>
-      <c r="K11" s="182" t="n"/>
-      <c r="L11" s="182" t="n"/>
-      <c r="M11" s="182" t="n"/>
-      <c r="N11" s="182" t="n"/>
-      <c r="O11" s="182" t="n"/>
+      <c r="H11" s="182" t="n">
+        <v>4260</v>
+      </c>
+      <c r="I11" s="182" t="n">
+        <v>4260</v>
+      </c>
+      <c r="J11" s="182" t="n">
+        <v>3811</v>
+      </c>
+      <c r="K11" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="182" t="n">
+        <v>437</v>
+      </c>
+      <c r="M11" s="182" t="n">
+        <v>12</v>
+      </c>
+      <c r="N11" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="182" t="n">
+        <v>34746</v>
+      </c>
       <c r="P11" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q11" s="86" t="n"/>
+      <c r="Q11" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 21 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="24" customHeight="1" s="80">
       <c r="A12" s="177" t="n">

</xml_diff>

<commit_message>
feat: update crawl 27/8
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -10182,7 +10182,7 @@
         <v>46260.022528125</v>
       </c>
       <c r="F12" s="180" t="n">
-        <v>46260.69894597779</v>
+        <v>46260.69894597222</v>
       </c>
       <c r="G12" s="181">
         <f>IF(OR(E12="",F12=""),"",(F12-E12)*24)</f>
@@ -10232,27 +10232,56 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E13" s="180" t="n"/>
-      <c r="F13" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="E13" s="180" t="n">
+        <v>46261.02233122685</v>
+      </c>
+      <c r="F13" s="180" t="n">
+        <v>46261.77158122685</v>
+      </c>
       <c r="G13" s="181">
         <f>IF(OR(E13="",F13=""),"",(F13-E13)*24)</f>
         <v/>
       </c>
-      <c r="H13" s="182" t="n"/>
-      <c r="I13" s="182" t="n"/>
-      <c r="J13" s="182" t="n"/>
-      <c r="K13" s="182" t="n"/>
-      <c r="L13" s="182" t="n"/>
-      <c r="M13" s="182" t="n"/>
-      <c r="N13" s="182" t="n"/>
-      <c r="O13" s="182" t="n"/>
+      <c r="H13" s="182" t="n">
+        <v>4260</v>
+      </c>
+      <c r="I13" s="182" t="n">
+        <v>4260</v>
+      </c>
+      <c r="J13" s="182" t="n">
+        <v>3747</v>
+      </c>
+      <c r="K13" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="182" t="n">
+        <v>405</v>
+      </c>
+      <c r="M13" s="182" t="n">
+        <v>84</v>
+      </c>
+      <c r="N13" s="182" t="n">
+        <v>24</v>
+      </c>
+      <c r="O13" s="182" t="n">
+        <v>33540</v>
+      </c>
       <c r="P13" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q13" s="86" t="n"/>
+      <c r="Q13" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 23 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="24" customHeight="1" s="80">
       <c r="A14" s="177" t="n">
@@ -10265,10 +10294,17 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E14" s="180" t="n"/>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="E14" s="180" t="n">
+        <v>46262.02246919833</v>
+      </c>
       <c r="F14" s="180" t="n"/>
       <c r="G14" s="181">
         <f>IF(OR(E14="",F14=""),"",(F14-E14)*24)</f>
@@ -10285,7 +10321,11 @@
       <c r="P14" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q14" s="86" t="n"/>
+      <c r="Q14" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled crawl đã tạo durable run; save_artifacts=false</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="24" customHeight="1" s="80">
       <c r="A15" s="177" t="n">

</xml_diff>

<commit_message>
feat: update crawl 28/8
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -10294,7 +10294,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Đang chạy</t>
+          <t>Hoàn thành có lỗi</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -10303,27 +10303,45 @@
         </is>
       </c>
       <c r="E14" s="180" t="n">
-        <v>46262.02246919833</v>
-      </c>
-      <c r="F14" s="180" t="n"/>
+        <v>46262.02246920139</v>
+      </c>
+      <c r="F14" s="180" t="n">
+        <v>46262.69405218779</v>
+      </c>
       <c r="G14" s="181">
         <f>IF(OR(E14="",F14=""),"",(F14-E14)*24)</f>
         <v/>
       </c>
-      <c r="H14" s="182" t="n"/>
-      <c r="I14" s="182" t="n"/>
-      <c r="J14" s="182" t="n"/>
-      <c r="K14" s="182" t="n"/>
-      <c r="L14" s="182" t="n"/>
-      <c r="M14" s="182" t="n"/>
-      <c r="N14" s="182" t="n"/>
-      <c r="O14" s="182" t="n"/>
+      <c r="H14" s="182" t="n">
+        <v>4260</v>
+      </c>
+      <c r="I14" s="182" t="n">
+        <v>4260</v>
+      </c>
+      <c r="J14" s="182" t="n">
+        <v>3768</v>
+      </c>
+      <c r="K14" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="182" t="n">
+        <v>384</v>
+      </c>
+      <c r="M14" s="182" t="n">
+        <v>96</v>
+      </c>
+      <c r="N14" s="182" t="n">
+        <v>12</v>
+      </c>
+      <c r="O14" s="182" t="n">
+        <v>34100</v>
+      </c>
       <c r="P14" s="182" t="n">
         <v>12</v>
       </c>
       <c r="Q14" s="86" t="inlineStr">
         <is>
-          <t>Scheduled crawl đã tạo durable run; save_artifacts=false</t>
+          <t>Scheduled run 24 đã đạt terminal state</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: update crawl 29/8
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -10306,7 +10306,7 @@
         <v>46262.02246920139</v>
       </c>
       <c r="F14" s="180" t="n">
-        <v>46262.69405218779</v>
+        <v>46262.6940521875</v>
       </c>
       <c r="G14" s="181">
         <f>IF(OR(E14="",F14=""),"",(F14-E14)*24)</f>
@@ -10356,27 +10356,56 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E15" s="180" t="n"/>
-      <c r="F15" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="E15" s="180" t="n">
+        <v>46263.02209759259</v>
+      </c>
+      <c r="F15" s="180" t="n">
+        <v>46263.69990558667</v>
+      </c>
       <c r="G15" s="181">
         <f>IF(OR(E15="",F15=""),"",(F15-E15)*24)</f>
         <v/>
       </c>
-      <c r="H15" s="182" t="n"/>
-      <c r="I15" s="182" t="n"/>
-      <c r="J15" s="182" t="n"/>
-      <c r="K15" s="182" t="n"/>
-      <c r="L15" s="182" t="n"/>
-      <c r="M15" s="182" t="n"/>
-      <c r="N15" s="182" t="n"/>
-      <c r="O15" s="182" t="n"/>
+      <c r="H15" s="182" t="n">
+        <v>4260</v>
+      </c>
+      <c r="I15" s="182" t="n">
+        <v>4260</v>
+      </c>
+      <c r="J15" s="182" t="n">
+        <v>3755</v>
+      </c>
+      <c r="K15" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="182" t="n">
+        <v>409</v>
+      </c>
+      <c r="M15" s="182" t="n">
+        <v>84</v>
+      </c>
+      <c r="N15" s="182" t="n">
+        <v>12</v>
+      </c>
+      <c r="O15" s="182" t="n">
+        <v>33683</v>
+      </c>
       <c r="P15" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q15" s="86" t="n"/>
+      <c r="Q15" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 25 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="24" customHeight="1" s="80">
       <c r="A16" s="177" t="n">

</xml_diff>

<commit_message>
feat: update crawl 30/8
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -10368,7 +10368,7 @@
         <v>46263.02209759259</v>
       </c>
       <c r="F15" s="180" t="n">
-        <v>46263.69990558667</v>
+        <v>46263.69990559028</v>
       </c>
       <c r="G15" s="181">
         <f>IF(OR(E15="",F15=""),"",(F15-E15)*24)</f>
@@ -10418,27 +10418,56 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E16" s="180" t="n"/>
-      <c r="F16" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="E16" s="180" t="n">
+        <v>46264.02248944445</v>
+      </c>
+      <c r="F16" s="180" t="n">
+        <v>46264.70586725581</v>
+      </c>
       <c r="G16" s="181">
         <f>IF(OR(E16="",F16=""),"",(F16-E16)*24)</f>
         <v/>
       </c>
-      <c r="H16" s="182" t="n"/>
-      <c r="I16" s="182" t="n"/>
-      <c r="J16" s="182" t="n"/>
-      <c r="K16" s="182" t="n"/>
-      <c r="L16" s="182" t="n"/>
-      <c r="M16" s="182" t="n"/>
-      <c r="N16" s="182" t="n"/>
-      <c r="O16" s="182" t="n"/>
+      <c r="H16" s="182" t="n">
+        <v>4260</v>
+      </c>
+      <c r="I16" s="182" t="n">
+        <v>4260</v>
+      </c>
+      <c r="J16" s="182" t="n">
+        <v>3853</v>
+      </c>
+      <c r="K16" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="182" t="n">
+        <v>323</v>
+      </c>
+      <c r="M16" s="182" t="n">
+        <v>72</v>
+      </c>
+      <c r="N16" s="182" t="n">
+        <v>12</v>
+      </c>
+      <c r="O16" s="182" t="n">
+        <v>35199</v>
+      </c>
       <c r="P16" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q16" s="86" t="n"/>
+      <c r="Q16" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 26 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="24" customHeight="1" s="80">
       <c r="A17" s="177" t="n">

</xml_diff>

<commit_message>
feat: update crawl 31/8
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -10430,7 +10430,7 @@
         <v>46264.02248944445</v>
       </c>
       <c r="F16" s="180" t="n">
-        <v>46264.70586725581</v>
+        <v>46264.70586725695</v>
       </c>
       <c r="G16" s="181">
         <f>IF(OR(E16="",F16=""),"",(F16-E16)*24)</f>
@@ -10480,27 +10480,56 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E17" s="180" t="n"/>
-      <c r="F17" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="E17" s="180" t="n">
+        <v>46265.02229482639</v>
+      </c>
+      <c r="F17" s="180" t="n">
+        <v>46265.69593640573</v>
+      </c>
       <c r="G17" s="181">
         <f>IF(OR(E17="",F17=""),"",(F17-E17)*24)</f>
         <v/>
       </c>
-      <c r="H17" s="182" t="n"/>
-      <c r="I17" s="182" t="n"/>
-      <c r="J17" s="182" t="n"/>
-      <c r="K17" s="182" t="n"/>
-      <c r="L17" s="182" t="n"/>
-      <c r="M17" s="182" t="n"/>
-      <c r="N17" s="182" t="n"/>
-      <c r="O17" s="182" t="n"/>
+      <c r="H17" s="182" t="n">
+        <v>4260</v>
+      </c>
+      <c r="I17" s="182" t="n">
+        <v>4260</v>
+      </c>
+      <c r="J17" s="182" t="n">
+        <v>3858</v>
+      </c>
+      <c r="K17" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="182" t="n">
+        <v>318</v>
+      </c>
+      <c r="M17" s="182" t="n">
+        <v>72</v>
+      </c>
+      <c r="N17" s="182" t="n">
+        <v>12</v>
+      </c>
+      <c r="O17" s="182" t="n">
+        <v>34469</v>
+      </c>
       <c r="P17" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q17" s="86" t="n"/>
+      <c r="Q17" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 27 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="24" customHeight="1" s="80">
       <c r="A18" s="177" t="n">

</xml_diff>

<commit_message>
feat: update crawl 1/9
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -10492,7 +10492,7 @@
         <v>46265.02229482639</v>
       </c>
       <c r="F17" s="180" t="n">
-        <v>46265.69593640573</v>
+        <v>46265.69593640047</v>
       </c>
       <c r="G17" s="181">
         <f>IF(OR(E17="",F17=""),"",(F17-E17)*24)</f>
@@ -10542,27 +10542,56 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E18" s="180" t="n"/>
-      <c r="F18" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="E18" s="180" t="n">
+        <v>46266.02162206019</v>
+      </c>
+      <c r="F18" s="180" t="n">
+        <v>46266.69667009647</v>
+      </c>
       <c r="G18" s="181">
         <f>IF(OR(E18="",F18=""),"",(F18-E18)*24)</f>
         <v/>
       </c>
-      <c r="H18" s="182" t="n"/>
-      <c r="I18" s="182" t="n"/>
-      <c r="J18" s="182" t="n"/>
-      <c r="K18" s="182" t="n"/>
-      <c r="L18" s="182" t="n"/>
-      <c r="M18" s="182" t="n"/>
-      <c r="N18" s="182" t="n"/>
-      <c r="O18" s="182" t="n"/>
+      <c r="H18" s="182" t="n">
+        <v>4260</v>
+      </c>
+      <c r="I18" s="182" t="n">
+        <v>4260</v>
+      </c>
+      <c r="J18" s="182" t="n">
+        <v>3862</v>
+      </c>
+      <c r="K18" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="182" t="n">
+        <v>314</v>
+      </c>
+      <c r="M18" s="182" t="n">
+        <v>72</v>
+      </c>
+      <c r="N18" s="182" t="n">
+        <v>12</v>
+      </c>
+      <c r="O18" s="182" t="n">
+        <v>34376</v>
+      </c>
       <c r="P18" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q18" s="86" t="n"/>
+      <c r="Q18" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 28 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="24" customHeight="1" s="80">
       <c r="A19" s="177" t="n">

</xml_diff>

<commit_message>
feat: update crawl 2/9
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -10604,7 +10604,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Đang chạy</t>
+          <t>Hoàn thành có lỗi</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -10613,27 +10613,45 @@
         </is>
       </c>
       <c r="E19" s="180" t="n">
-        <v>46267.02152130967</v>
-      </c>
-      <c r="F19" s="180" t="n"/>
+        <v>46267.02152130787</v>
+      </c>
+      <c r="F19" s="180" t="n">
+        <v>46267.89147708264</v>
+      </c>
       <c r="G19" s="181">
         <f>IF(OR(E19="",F19=""),"",(F19-E19)*24)</f>
         <v/>
       </c>
-      <c r="H19" s="182" t="n"/>
-      <c r="I19" s="182" t="n"/>
-      <c r="J19" s="182" t="n"/>
-      <c r="K19" s="182" t="n"/>
-      <c r="L19" s="182" t="n"/>
-      <c r="M19" s="182" t="n"/>
-      <c r="N19" s="182" t="n"/>
-      <c r="O19" s="182" t="n"/>
+      <c r="H19" s="182" t="n">
+        <v>4260</v>
+      </c>
+      <c r="I19" s="182" t="n">
+        <v>4260</v>
+      </c>
+      <c r="J19" s="182" t="n">
+        <v>3853</v>
+      </c>
+      <c r="K19" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="182" t="n">
+        <v>323</v>
+      </c>
+      <c r="M19" s="182" t="n">
+        <v>72</v>
+      </c>
+      <c r="N19" s="182" t="n">
+        <v>12</v>
+      </c>
+      <c r="O19" s="182" t="n">
+        <v>34019</v>
+      </c>
       <c r="P19" s="182" t="n">
         <v>12</v>
       </c>
       <c r="Q19" s="86" t="inlineStr">
         <is>
-          <t>Scheduled crawl đã tạo durable run; save_artifacts=false</t>
+          <t>Scheduled run 29 đã đạt terminal state</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: update crawl 4/9
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -10616,7 +10616,7 @@
         <v>46267.02152130787</v>
       </c>
       <c r="F19" s="180" t="n">
-        <v>46267.89147708264</v>
+        <v>46267.89147708334</v>
       </c>
       <c r="G19" s="181">
         <f>IF(OR(E19="",F19=""),"",(F19-E19)*24)</f>
@@ -10666,27 +10666,56 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E20" s="180" t="n"/>
-      <c r="F20" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="E20" s="180" t="n">
+        <v>46268.02163693287</v>
+      </c>
+      <c r="F20" s="180" t="n">
+        <v>46269.06629293165</v>
+      </c>
       <c r="G20" s="181">
         <f>IF(OR(E20="",F20=""),"",(F20-E20)*24)</f>
         <v/>
       </c>
-      <c r="H20" s="182" t="n"/>
-      <c r="I20" s="182" t="n"/>
-      <c r="J20" s="182" t="n"/>
-      <c r="K20" s="182" t="n"/>
-      <c r="L20" s="182" t="n"/>
-      <c r="M20" s="182" t="n"/>
-      <c r="N20" s="182" t="n"/>
-      <c r="O20" s="182" t="n"/>
+      <c r="H20" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I20" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J20" s="182" t="n">
+        <v>3867</v>
+      </c>
+      <c r="K20" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="182" t="n">
+        <v>309</v>
+      </c>
+      <c r="M20" s="182" t="n">
+        <v>48</v>
+      </c>
+      <c r="N20" s="182" t="n">
+        <v>24</v>
+      </c>
+      <c r="O20" s="182" t="n">
+        <v>35445</v>
+      </c>
       <c r="P20" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q20" s="86" t="n"/>
+      <c r="Q20" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 30 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="24" customHeight="1" s="80">
       <c r="A21" s="177" t="n">

</xml_diff>

<commit_message>
feat: update crawl 6/9
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -10802,7 +10802,7 @@
         <v>46270.02194637732</v>
       </c>
       <c r="F22" s="180" t="n">
-        <v>46270.84142836356</v>
+        <v>46270.84142836805</v>
       </c>
       <c r="G22" s="181">
         <f>IF(OR(E22="",F22=""),"",(F22-E22)*24)</f>
@@ -10852,27 +10852,56 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E23" s="180" t="n"/>
-      <c r="F23" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="E23" s="180" t="n">
+        <v>46271.02241783565</v>
+      </c>
+      <c r="F23" s="180" t="n">
+        <v>46271.83497188657</v>
+      </c>
       <c r="G23" s="181">
         <f>IF(OR(E23="",F23=""),"",(F23-E23)*24)</f>
         <v/>
       </c>
-      <c r="H23" s="182" t="n"/>
-      <c r="I23" s="182" t="n"/>
-      <c r="J23" s="182" t="n"/>
-      <c r="K23" s="182" t="n"/>
-      <c r="L23" s="182" t="n"/>
-      <c r="M23" s="182" t="n"/>
-      <c r="N23" s="182" t="n"/>
-      <c r="O23" s="182" t="n"/>
+      <c r="H23" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I23" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J23" s="182" t="n">
+        <v>3851</v>
+      </c>
+      <c r="K23" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" s="182" t="n">
+        <v>337</v>
+      </c>
+      <c r="M23" s="182" t="n">
+        <v>36</v>
+      </c>
+      <c r="N23" s="182" t="n">
+        <v>24</v>
+      </c>
+      <c r="O23" s="182" t="n">
+        <v>34793</v>
+      </c>
       <c r="P23" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q23" s="86" t="n"/>
+      <c r="Q23" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 33 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="24" customHeight="1" s="80">
       <c r="A24" s="177" t="n">
@@ -10885,10 +10914,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E24" s="180" t="n"/>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="E24" s="180" t="n">
+        <v>46272.02219992066</v>
+      </c>
       <c r="F24" s="180" t="n"/>
       <c r="G24" s="181">
         <f>IF(OR(E24="",F24=""),"",(F24-E24)*24)</f>
@@ -10905,7 +10941,11 @@
       <c r="P24" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q24" s="86" t="n"/>
+      <c r="Q24" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled crawl đã tạo durable run; save_artifacts=false</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="24" customHeight="1" s="80">
       <c r="A25" s="177" t="n">

</xml_diff>

<commit_message>
feat: update crawl 7/9
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -10914,7 +10914,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Đang chạy</t>
+          <t>Hoàn thành có lỗi</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -10923,27 +10923,45 @@
         </is>
       </c>
       <c r="E24" s="180" t="n">
-        <v>46272.02219992066</v>
-      </c>
-      <c r="F24" s="180" t="n"/>
+        <v>46272.02219991898</v>
+      </c>
+      <c r="F24" s="180" t="n">
+        <v>46272.83890384883</v>
+      </c>
       <c r="G24" s="181">
         <f>IF(OR(E24="",F24=""),"",(F24-E24)*24)</f>
         <v/>
       </c>
-      <c r="H24" s="182" t="n"/>
-      <c r="I24" s="182" t="n"/>
-      <c r="J24" s="182" t="n"/>
-      <c r="K24" s="182" t="n"/>
-      <c r="L24" s="182" t="n"/>
-      <c r="M24" s="182" t="n"/>
-      <c r="N24" s="182" t="n"/>
-      <c r="O24" s="182" t="n"/>
+      <c r="H24" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I24" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J24" s="182" t="n">
+        <v>3853</v>
+      </c>
+      <c r="K24" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" s="182" t="n">
+        <v>335</v>
+      </c>
+      <c r="M24" s="182" t="n">
+        <v>36</v>
+      </c>
+      <c r="N24" s="182" t="n">
+        <v>24</v>
+      </c>
+      <c r="O24" s="182" t="n">
+        <v>35350</v>
+      </c>
       <c r="P24" s="182" t="n">
         <v>12</v>
       </c>
       <c r="Q24" s="86" t="inlineStr">
         <is>
-          <t>Scheduled crawl đã tạo durable run; save_artifacts=false</t>
+          <t>Scheduled run 34 đã đạt terminal state</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: update crawl 9/9
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -10926,7 +10926,7 @@
         <v>46272.02219991898</v>
       </c>
       <c r="F24" s="180" t="n">
-        <v>46272.83890384883</v>
+        <v>46272.83890385416</v>
       </c>
       <c r="G24" s="181">
         <f>IF(OR(E24="",F24=""),"",(F24-E24)*24)</f>
@@ -10976,27 +10976,56 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E25" s="180" t="n"/>
-      <c r="F25" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="E25" s="180" t="n">
+        <v>46273.02228375</v>
+      </c>
+      <c r="F25" s="180" t="n">
+        <v>46273.84941858138</v>
+      </c>
       <c r="G25" s="181">
         <f>IF(OR(E25="",F25=""),"",(F25-E25)*24)</f>
         <v/>
       </c>
-      <c r="H25" s="182" t="n"/>
-      <c r="I25" s="182" t="n"/>
-      <c r="J25" s="182" t="n"/>
-      <c r="K25" s="182" t="n"/>
-      <c r="L25" s="182" t="n"/>
-      <c r="M25" s="182" t="n"/>
-      <c r="N25" s="182" t="n"/>
-      <c r="O25" s="182" t="n"/>
+      <c r="H25" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I25" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J25" s="182" t="n">
+        <v>3842</v>
+      </c>
+      <c r="K25" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" s="182" t="n">
+        <v>334</v>
+      </c>
+      <c r="M25" s="182" t="n">
+        <v>48</v>
+      </c>
+      <c r="N25" s="182" t="n">
+        <v>24</v>
+      </c>
+      <c r="O25" s="182" t="n">
+        <v>34326</v>
+      </c>
       <c r="P25" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q25" s="86" t="n"/>
+      <c r="Q25" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 35 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="24" customHeight="1" s="80">
       <c r="A26" s="177" t="n">

</xml_diff>

<commit_message>
feat: update crawl 11/9
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SUMMARY" sheetId="1" r:id="R1634e374f4514649"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DAILY_CRAWL_PLAN" sheetId="2" r:id="R44812168e02143ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CRAWL_LOG" sheetId="3" r:id="R917457e6b1674af1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SLOT_RULES" sheetId="4" r:id="Read77a6e86b54b1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AUTOMATION_CONFIG" sheetId="5" r:id="Rad235b620e264f6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="6" r:id="R9df59ce8d87e4a8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SUMMARY" sheetId="1" r:id="R54fe58e31f08495c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DAILY_CRAWL_PLAN" sheetId="2" r:id="R3cdb8accfe7749a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CRAWL_LOG" sheetId="3" r:id="R97817e3b59e54739"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SLOT_RULES" sheetId="4" r:id="R9fbcac87a4a74ff9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AUTOMATION_CONFIG" sheetId="5" r:id="R17b9984c950c4253"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="6" r:id="R5c5f4a45d25e4dfe"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1229,7 +1229,7 @@
       </x:c>
       <x:c r="B10" s="175" t="n">
         <x:f>COUNTIF('CRAWL_LOG'!$C$4:$C$108,"Hoàn thành có lỗi")</x:f>
-        <x:v>14</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1240,7 +1240,7 @@
       </x:c>
       <x:c r="B11" s="175" t="n">
         <x:f>COUNTIF('CRAWL_LOG'!$C$4:$C$108,"Đang chạy")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -1251,7 +1251,7 @@
       </x:c>
       <x:c r="B12" s="176" t="n">
         <x:f>COUNTIF('CRAWL_LOG'!$C$4:$C$108,"Chưa chạy")</x:f>
-        <x:v>81</x:v>
+        <x:v>80</x:v>
       </x:c>
     </x:row>
     <x:row r="15" s="80" customFormat="1" ht="35" customHeight="1">
@@ -3186,7 +3186,7 @@
       </x:c>
       <x:c r="T26" s="125" t="str">
         <x:f>'CRAWL_LOG'!C26</x:f>
-        <x:v>Đang chạy</x:v>
+        <x:v>Hoàn thành có lỗi</x:v>
       </x:c>
       <x:c r="U26" s="86" t="inlineStr">
         <x:is>
@@ -3340,7 +3340,7 @@
       </x:c>
       <x:c r="T28" s="125" t="str">
         <x:f>'CRAWL_LOG'!C28</x:f>
-        <x:v>Chưa chạy</x:v>
+        <x:v>Hoàn thành có lỗi</x:v>
       </x:c>
       <x:c r="U28" s="86" t="inlineStr">
         <x:is>
@@ -9521,7 +9521,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a59b0d596aa4ef2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R770b92b95c4a4d01"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11023,38 +11023,51 @@
           <x:t xml:space="preserve">00:30</x:t>
         </x:is>
       </x:c>
-      <x:c r="C26" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Đang chạy</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D26" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">36</x:t>
-        </x:is>
+      <x:c r="C26" t="str">
+        <x:v>Hoàn thành có lỗi</x:v>
+      </x:c>
+      <x:c r="D26" t="n">
+        <x:v>36</x:v>
       </x:c>
       <x:c r="E26" s="180" t="n">
-        <x:v>46274.02166638889</x:v>
-      </x:c>
-      <x:c r="F26" s="180" t="n"/>
-      <x:c r="G26" s="181" t="str">
+        <x:v>46274.021689814814</x:v>
+      </x:c>
+      <x:c r="F26" s="180" t="n">
+        <x:v>46275.16547453703</x:v>
+      </x:c>
+      <x:c r="G26" s="181" t="n">
         <x:f>IF(OR(E26="",F26=""),"",(F26-E26)*24)</x:f>
-      </x:c>
-      <x:c r="H26" s="182" t="n"/>
-      <x:c r="I26" s="182" t="n"/>
-      <x:c r="J26" s="182" t="n"/>
-      <x:c r="K26" s="182" t="n"/>
-      <x:c r="L26" s="182" t="n"/>
-      <x:c r="M26" s="182" t="n"/>
-      <x:c r="N26" s="182" t="n"/>
-      <x:c r="O26" s="182" t="n"/>
+        <x:v>27.450833333248738</x:v>
+      </x:c>
+      <x:c r="H26" s="182" t="n">
+        <x:v>4248</x:v>
+      </x:c>
+      <x:c r="I26" s="182" t="n">
+        <x:v>4248</x:v>
+      </x:c>
+      <x:c r="J26" s="182" t="n">
+        <x:v>3713</x:v>
+      </x:c>
+      <x:c r="K26" s="182" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L26" s="182" t="n">
+        <x:v>382</x:v>
+      </x:c>
+      <x:c r="M26" s="182" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="N26" s="182" t="n">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="O26" s="182" t="n">
+        <x:v>33440</x:v>
+      </x:c>
       <x:c r="P26" s="182" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="Q26" s="86" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Scheduled crawl đã tạo durable run; save_artifacts=false</x:t>
-        </x:is>
+      <x:c r="Q26" s="86" t="str">
+        <x:v>Scheduled run 36 đã đạt terminal state; save_artifacts=false; scraper_version=2.3.0</x:v>
       </x:c>
     </x:row>
     <x:row r="27" s="80" customFormat="1" ht="24" customHeight="1">
@@ -11066,8 +11079,10 @@
           <x:t xml:space="preserve">00:30</x:t>
         </x:is>
       </x:c>
-      <x:c r="C27" t="str">
-        <x:v>Hoàn thành có lỗi</x:v>
+      <x:c r="C27" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Hoàn thành có lỗi</x:t>
+        </x:is>
       </x:c>
       <x:c r="D27" t="inlineStr">
         <x:is>
@@ -11075,14 +11090,14 @@
         </x:is>
       </x:c>
       <x:c r="E27" s="180" t="n">
-        <x:v>46275.166134259256</x:v>
+        <x:v>46275.16613425926</x:v>
       </x:c>
       <x:c r="F27" s="180" t="n">
         <x:v>46275.98001157407</x:v>
       </x:c>
       <x:c r="G27" s="181" t="n">
         <x:f>IF(OR(E27="",F27=""),"",(F27-E27)*24)</x:f>
-        <x:v>19.533055555599276</x:v>
+        <x:v>19.533055555424653</x:v>
       </x:c>
       <x:c r="H27" s="182" t="n">
         <x:v>4248</x:v>
@@ -11111,8 +11126,10 @@
       <x:c r="P27" s="182" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="Q27" s="86" t="str">
-        <x:v>Scheduled run 37 đã đạt terminal state; save_artifacts=false; scraper_version=2.3.0</x:v>
+      <x:c r="Q27" s="86" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Scheduled run 37 đã đạt terminal state; save_artifacts=false; scraper_version=2.3.0</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="28" s="80" customFormat="1" ht="24" customHeight="1">
@@ -11126,26 +11143,56 @@
       </x:c>
       <x:c r="C28" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Chưa chạy</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E28" s="180" t="n"/>
-      <x:c r="F28" s="180" t="n"/>
-      <x:c r="G28" s="181" t="str">
+          <x:t xml:space="preserve">Hoàn thành có lỗi</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D28" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">38</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E28" s="180" t="n">
+        <x:v>46276.0233637037</x:v>
+      </x:c>
+      <x:c r="F28" s="180" t="n">
+        <x:v>46276.85465078014</x:v>
+      </x:c>
+      <x:c r="G28" s="181" t="n">
         <x:f>IF(OR(E28="",F28=""),"",(F28-E28)*24)</x:f>
-      </x:c>
-      <x:c r="H28" s="182" t="n"/>
-      <x:c r="I28" s="182" t="n"/>
-      <x:c r="J28" s="182" t="n"/>
-      <x:c r="K28" s="182" t="n"/>
-      <x:c r="L28" s="182" t="n"/>
-      <x:c r="M28" s="182" t="n"/>
-      <x:c r="N28" s="182" t="n"/>
-      <x:c r="O28" s="182" t="n"/>
+        <x:v>19.950889834435657</x:v>
+      </x:c>
+      <x:c r="H28" s="182" t="n">
+        <x:v>4248</x:v>
+      </x:c>
+      <x:c r="I28" s="182" t="n">
+        <x:v>4248</x:v>
+      </x:c>
+      <x:c r="J28" s="182" t="n">
+        <x:v>3822</x:v>
+      </x:c>
+      <x:c r="K28" s="182" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L28" s="182" t="n">
+        <x:v>366</x:v>
+      </x:c>
+      <x:c r="M28" s="182" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="N28" s="182" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="O28" s="182" t="n">
+        <x:v>34224</x:v>
+      </x:c>
       <x:c r="P28" s="182" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="Q28" s="86" t="n"/>
+      <x:c r="Q28" s="86" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Scheduled run 38 đã đạt terminal state</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="29" s="80" customFormat="1" ht="24" customHeight="1">
       <x:c r="A29" s="177" t="n">
@@ -13727,7 +13774,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbcd403a9627d4290"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37386d5a855149d9"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>